<commit_message>
ZRU : corriger xlsx.ts pour les attributs de cellule en ordre quelconque et indexation des lignes
Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/lib/zru/__fixtures__/mini.xlsx
+++ b/src/lib/zru/__fixtures__/mini.xlsx
@@ -23,6 +23,9 @@
   </si>
   <si>
     <t>⁽²⁾</t>
+  </si>
+  <si>
+    <t>StyleCell</t>
   </si>
 </sst>
 </file>
@@ -65,6 +68,12 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c s="3" r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6"/>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>